<commit_message>
feat: implement high value DD office note wizard with PDF generation and regional auto-fill
</commit_message>
<xml_diff>
--- a/ro_workstation/data/mis/archive/20250331.xlsx
+++ b/ro_workstation/data/mis/archive/20250331.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24827"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,24 +8,33 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Daily_MIS\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9927B8F-7613-4830-951C-229119FC1C18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6526D900-6A5A-4011-AE19-D0E4288D33B4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>S No</t>
   </si>
@@ -104,6 +113,33 @@
   <si>
     <t>ADV</t>
   </si>
+  <si>
+    <t>Cash on Hand</t>
+  </si>
+  <si>
+    <t>ATM Cash</t>
+  </si>
+  <si>
+    <t>BC Cash</t>
+  </si>
+  <si>
+    <t>BNA Cash</t>
+  </si>
+  <si>
+    <t>Total Cash</t>
+  </si>
+  <si>
+    <t>CRL</t>
+  </si>
+  <si>
+    <t>Excess</t>
+  </si>
+  <si>
+    <t>Bulk Dep</t>
+  </si>
+  <si>
+    <t>PL</t>
+  </si>
 </sst>
 </file>
 
@@ -113,7 +149,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="0000"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,14 +158,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color theme="1" tint="0.0499899983406067"/>
+      <color theme="1" tint="4.9989318521683403E-2"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -159,130 +189,38 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color indexed="64"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment/>
-      <protection/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="15" builtinId="5"/>
-    <cellStyle name="Currency" xfId="16" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="17" builtinId="7"/>
-    <cellStyle name="Comma" xfId="18" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="19" builtinId="6"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -590,37 +528,37 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEF409BC-5808-478A-B6BA-9A096C89F648}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEF409BC-5808-478A-B6BA-9A096C89F648}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:AW56"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:AI57"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="5" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5714285714286" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.2857142857143" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.1428571428571" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.4285714285714" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.2857142857143" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.2857142857143" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.8571428571429" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10" bestFit="1" customWidth="1"/>
     <col min="17" max="18" width="9" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.8571428571429" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.7142857142857" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.2857142857143" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="9" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.5714285714286" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="9" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="10" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.5714285714286" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="15">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -699,8 +637,35 @@
       <c r="Z1" s="3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:49" ht="15">
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -723,7 +688,7 @@
         <v>2100.8020761590005</v>
       </c>
       <c r="H2" s="4">
-        <v>165.019990068</v>
+        <v>165.19991855200001</v>
       </c>
       <c r="I2" s="4">
         <v>24.359885379999994</v>
@@ -744,40 +709,40 @@
         <v>62.639514868000006</v>
       </c>
       <c r="O2" s="4">
-        <v>564.45099191400004</v>
+        <v>564.63092039800017</v>
       </c>
       <c r="P2" s="4">
-        <v>112.51059410900002</v>
+        <v>112.96952676800004</v>
       </c>
       <c r="Q2" s="4">
-        <v>38.765012959999986</v>
+        <v>38.861679235999979</v>
       </c>
       <c r="R2" s="4">
-        <v>15.866799371999997</v>
+        <v>15.841799108</v>
       </c>
       <c r="S2" s="4">
-        <v>1.531451712</v>
+        <v>0</v>
       </c>
       <c r="T2" s="4">
-        <v>18.812239549000001</v>
+        <v>28.685651296</v>
       </c>
       <c r="U2" s="4">
         <v>91.048242952999999</v>
       </c>
       <c r="V2" s="4">
-        <v>28.413291562999998</v>
+        <v>36.782932031000001</v>
       </c>
       <c r="W2" s="4">
-        <v>1004.4168570310001</v>
+        <v>1004.416857037</v>
       </c>
       <c r="X2" s="4">
         <v>68.025621167999986</v>
       </c>
       <c r="Y2" s="4">
-        <v>919.72681867799997</v>
+        <v>919.72681867399979</v>
       </c>
       <c r="Z2" s="4">
-        <v>2689.3209535199999</v>
+        <v>2697.6905943119996</v>
       </c>
       <c r="AA2" s="6"/>
       <c r="AB2" s="6"/>
@@ -788,22 +753,8 @@
       <c r="AG2" s="6"/>
       <c r="AH2" s="6"/>
       <c r="AI2" s="6"/>
-      <c r="AJ2" s="6"/>
-      <c r="AK2" s="6"/>
-      <c r="AL2" s="6"/>
-      <c r="AM2" s="6"/>
-      <c r="AN2" s="6"/>
-      <c r="AO2" s="6"/>
-      <c r="AP2" s="6"/>
-      <c r="AQ2" s="6"/>
-      <c r="AR2" s="6"/>
-      <c r="AS2" s="6"/>
-      <c r="AT2" s="6"/>
-      <c r="AU2" s="6"/>
-      <c r="AV2" s="6"/>
-      <c r="AW2" s="6"/>
-    </row>
-    <row r="3" spans="1:26" ht="15">
+    </row>
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -826,7 +777,7 @@
         <v>5536.2450165</v>
       </c>
       <c r="H3" s="3">
-        <v>899.71429720000003</v>
+        <v>917.70714559999999</v>
       </c>
       <c r="I3" s="3">
         <v>96.453983199999996</v>
@@ -847,10 +798,10 @@
         <v>316.28346700000009</v>
       </c>
       <c r="O3" s="3">
-        <v>1868.8023799000009</v>
+        <v>1886.7952283000013</v>
       </c>
       <c r="P3" s="3">
-        <v>231.26827030000001</v>
+        <v>271.18860400000005</v>
       </c>
       <c r="Q3" s="3">
         <v>417.47477670000006</v>
@@ -862,28 +813,28 @@
         <v>0</v>
       </c>
       <c r="T3" s="3">
-        <v>22.841458700000004</v>
+        <v>108.01561539999985</v>
       </c>
       <c r="U3" s="3">
         <v>565.31906979999985</v>
       </c>
       <c r="V3" s="3">
-        <v>323.36340599999988</v>
+        <v>403.13070809999988</v>
       </c>
       <c r="W3" s="3">
-        <v>3598.3529410000001</v>
+        <v>3598.3529412000003</v>
       </c>
       <c r="X3" s="3">
         <v>245.6217278</v>
       </c>
       <c r="Y3" s="3">
-        <v>3270.9518560000001</v>
+        <v>3270.9518563000001</v>
       </c>
       <c r="Z3" s="3">
-        <v>7904.707617</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26" ht="15">
+        <v>7984.4750000000004</v>
+      </c>
+    </row>
+    <row r="4" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -939,10 +890,10 @@
         <v>106.8957355</v>
       </c>
       <c r="S4" s="3">
-        <v>1.0685133</v>
+        <v>0</v>
       </c>
       <c r="T4" s="3">
-        <v>17.505118899999999</v>
+        <v>19.610922199999965</v>
       </c>
       <c r="U4" s="3">
         <v>147.64750659999996</v>
@@ -951,7 +902,7 @@
         <v>122.55676469999999</v>
       </c>
       <c r="W4" s="3">
-        <v>2146.0299760000003</v>
+        <v>2146.0299763999997</v>
       </c>
       <c r="X4" s="3">
         <v>16.2842068</v>
@@ -960,10 +911,10 @@
         <v>2386.0642699999999</v>
       </c>
       <c r="Z4" s="3">
-        <v>3796.9017800000001</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" ht="15">
+        <v>3796.9017803000002</v>
+      </c>
+    </row>
+    <row r="5" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -1016,22 +967,22 @@
         <v>0</v>
       </c>
       <c r="R5" s="3">
-        <v>86.926729600000002</v>
+        <v>82.086133199999992</v>
       </c>
       <c r="S5" s="3">
         <v>0</v>
       </c>
       <c r="T5" s="3">
-        <v>27.781770500000004</v>
+        <v>62.150815900000033</v>
       </c>
       <c r="U5" s="3">
         <v>235.91020950000006</v>
       </c>
       <c r="V5" s="3">
-        <v>106.93487739999999</v>
+        <v>193.7675414</v>
       </c>
       <c r="W5" s="3">
-        <v>2316.3469559999999</v>
+        <v>2316.3469556999999</v>
       </c>
       <c r="X5" s="3">
         <v>269.26388320000001</v>
@@ -1040,10 +991,10 @@
         <v>1684.94496</v>
       </c>
       <c r="Z5" s="3">
-        <v>6244.3552749999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26" ht="15">
+        <v>6331.1880000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -1099,10 +1050,10 @@
         <v>15.964295100000001</v>
       </c>
       <c r="S6" s="3">
-        <v>3.7083369999999998</v>
+        <v>0</v>
       </c>
       <c r="T6" s="3">
-        <v>19.055186199999998</v>
+        <v>22.957943200000035</v>
       </c>
       <c r="U6" s="3">
         <v>366.11359180000005</v>
@@ -1111,7 +1062,7 @@
         <v>51.489972399999999</v>
       </c>
       <c r="W6" s="3">
-        <v>3493.880463</v>
+        <v>3493.8804632000001</v>
       </c>
       <c r="X6" s="3">
         <v>82.068611199999992</v>
@@ -1120,10 +1071,10 @@
         <v>2712.1499600000002</v>
       </c>
       <c r="Z6" s="3">
-        <v>5776.683266</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" ht="15">
+        <v>5776.6832655999997</v>
+      </c>
+    </row>
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -1182,7 +1133,7 @@
         <v>0</v>
       </c>
       <c r="T7" s="3">
-        <v>0.71033999999999997</v>
+        <v>12.837571899999977</v>
       </c>
       <c r="U7" s="3">
         <v>135.33099549999997</v>
@@ -1191,7 +1142,7 @@
         <v>65.915525400000007</v>
       </c>
       <c r="W7" s="3">
-        <v>1383.3506540000001</v>
+        <v>1383.3506542</v>
       </c>
       <c r="X7" s="3">
         <v>33.621768099999997</v>
@@ -1200,10 +1151,10 @@
         <v>659.20509650000008</v>
       </c>
       <c r="Z7" s="3">
-        <v>4609.7664610000002</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" ht="15">
+        <v>4609.7664612999997</v>
+      </c>
+    </row>
+    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -1259,10 +1210,10 @@
         <v>29.629866199999999</v>
       </c>
       <c r="S8" s="3">
-        <v>0.33871470000000004</v>
+        <v>0</v>
       </c>
       <c r="T8" s="3">
-        <v>41.187616399999996</v>
+        <v>49.9523163</v>
       </c>
       <c r="U8" s="3">
         <v>79.582182500000002</v>
@@ -1271,7 +1222,7 @@
         <v>17.138919000000001</v>
       </c>
       <c r="W8" s="3">
-        <v>1901.014408</v>
+        <v>1901.0144078000001</v>
       </c>
       <c r="X8" s="3">
         <v>114.43006440000001</v>
@@ -1280,10 +1231,10 @@
         <v>800.99790160000009</v>
       </c>
       <c r="Z8" s="3">
-        <v>3977.6644070000002</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26" ht="15">
+        <v>3977.6644065</v>
+      </c>
+    </row>
+    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -1339,10 +1290,10 @@
         <v>169.60852359999998</v>
       </c>
       <c r="S9" s="3">
-        <v>2.4683799999999998</v>
+        <v>0</v>
       </c>
       <c r="T9" s="3">
-        <v>24.972510100000001</v>
+        <v>64.698522500000095</v>
       </c>
       <c r="U9" s="3">
         <v>247.82848150000007</v>
@@ -1360,10 +1311,10 @@
         <v>2800.2052100000001</v>
       </c>
       <c r="Z9" s="3">
-        <v>5158.6444529999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:26" ht="15">
+        <v>5158.6444526000005</v>
+      </c>
+    </row>
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -1422,28 +1373,28 @@
         <v>0</v>
       </c>
       <c r="T10" s="3">
-        <v>737.39248850000001</v>
+        <v>906.44961760000012</v>
       </c>
       <c r="U10" s="3">
         <v>1573.9218116000002</v>
       </c>
       <c r="V10" s="3">
-        <v>216.3018922</v>
+        <v>857.73874310000008</v>
       </c>
       <c r="W10" s="3">
-        <v>5490.9791539999997</v>
+        <v>5490.9791542000003</v>
       </c>
       <c r="X10" s="3">
         <v>734.59108470000001</v>
       </c>
       <c r="Y10" s="3">
-        <v>5187.8496429999996</v>
+        <v>5187.8496433999999</v>
       </c>
       <c r="Z10" s="3">
-        <v>10623.06625</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" ht="15">
+        <v>11264.503000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -1499,10 +1450,10 @@
         <v>16.717104199999998</v>
       </c>
       <c r="S11" s="3">
-        <v>0.25190999999999997</v>
+        <v>0</v>
       </c>
       <c r="T11" s="3">
-        <v>3.2131545999999997</v>
+        <v>8.3561775000000509</v>
       </c>
       <c r="U11" s="3">
         <v>225.02662080000002</v>
@@ -1511,7 +1462,7 @@
         <v>55.866553899999985</v>
       </c>
       <c r="W11" s="3">
-        <v>7092.2012839999998</v>
+        <v>7092.2012838000001</v>
       </c>
       <c r="X11" s="3">
         <v>352.6824628</v>
@@ -1520,10 +1471,10 @@
         <v>8597.0364200000004</v>
       </c>
       <c r="Z11" s="3">
-        <v>7538.536301000001</v>
-      </c>
-    </row>
-    <row r="12" spans="1:26" ht="15">
+        <v>7538.5363006000007</v>
+      </c>
+    </row>
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -1582,7 +1533,7 @@
         <v>0</v>
       </c>
       <c r="T12" s="3">
-        <v>26.858680699999997</v>
+        <v>40.896978400000158</v>
       </c>
       <c r="U12" s="3">
         <v>927.75817370000016</v>
@@ -1591,7 +1542,7 @@
         <v>75.836092600000001</v>
       </c>
       <c r="W12" s="3">
-        <v>1841.4310210000001</v>
+        <v>1841.4310212</v>
       </c>
       <c r="X12" s="3">
         <v>40.760600400000001</v>
@@ -1600,10 +1551,10 @@
         <v>1419.44723</v>
       </c>
       <c r="Z12" s="3">
-        <v>5358.2559899999997</v>
-      </c>
-    </row>
-    <row r="13" spans="1:26" ht="15">
+        <v>5358.2559903000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -1659,10 +1610,10 @@
         <v>7.8223828999999991</v>
       </c>
       <c r="S13" s="3">
-        <v>2.2772188</v>
+        <v>0</v>
       </c>
       <c r="T13" s="3">
-        <v>17.153857200000001</v>
+        <v>42.779931800000007</v>
       </c>
       <c r="U13" s="3">
         <v>64.61907140000001</v>
@@ -1671,7 +1622,7 @@
         <v>30.127806800000002</v>
       </c>
       <c r="W13" s="3">
-        <v>2164.1722319999999</v>
+        <v>2164.1722322000001</v>
       </c>
       <c r="X13" s="3">
         <v>90.748328199999989</v>
@@ -1680,10 +1631,10 @@
         <v>1379.0155</v>
       </c>
       <c r="Z13" s="3">
-        <v>3369.6557329999996</v>
-      </c>
-    </row>
-    <row r="14" spans="1:26" ht="15">
+        <v>3369.6557330999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -1742,7 +1693,7 @@
         <v>0</v>
       </c>
       <c r="T14" s="3">
-        <v>34.389767599999999</v>
+        <v>35.470624499999985</v>
       </c>
       <c r="U14" s="3">
         <v>60.84895319999999</v>
@@ -1751,19 +1702,19 @@
         <v>12.645231599999999</v>
       </c>
       <c r="W14" s="3">
-        <v>1249.6069970000001</v>
+        <v>1249.6069974</v>
       </c>
       <c r="X14" s="3">
         <v>20.8246699</v>
       </c>
       <c r="Y14" s="3">
-        <v>2631.4991869999999</v>
+        <v>2631.4991871000002</v>
       </c>
       <c r="Z14" s="3">
-        <v>2856.6623960000002</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" ht="15">
+        <v>2856.6623959000003</v>
+      </c>
+    </row>
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -1819,10 +1770,10 @@
         <v>81.169736600000007</v>
       </c>
       <c r="S15" s="3">
-        <v>10.2104594</v>
+        <v>0</v>
       </c>
       <c r="T15" s="3">
-        <v>65.975355300000004</v>
+        <v>88.001417099999941</v>
       </c>
       <c r="U15" s="3">
         <v>261.62283479999996</v>
@@ -1831,7 +1782,7 @@
         <v>62.047302900000012</v>
       </c>
       <c r="W15" s="3">
-        <v>1741.7476220000001</v>
+        <v>1741.7476218000002</v>
       </c>
       <c r="X15" s="3">
         <v>118.40192739999999</v>
@@ -1840,10 +1791,10 @@
         <v>2749.1504399999999</v>
       </c>
       <c r="Z15" s="3">
-        <v>3907.5913800000003</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" ht="15">
+        <v>3907.5913794999997</v>
+      </c>
+    </row>
+    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -1899,10 +1850,10 @@
         <v>89.110698299999996</v>
       </c>
       <c r="S16" s="3">
-        <v>1.3158151</v>
+        <v>0</v>
       </c>
       <c r="T16" s="3">
-        <v>27.488212299999997</v>
+        <v>40.838054600000042</v>
       </c>
       <c r="U16" s="3">
         <v>299.58771590000003</v>
@@ -1920,10 +1871,10 @@
         <v>998.16579000000002</v>
       </c>
       <c r="Z16" s="3">
-        <v>8797.5654830000003</v>
-      </c>
-    </row>
-    <row r="17" spans="1:26" ht="15">
+        <v>8797.5654829000014</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -1982,7 +1933,7 @@
         <v>0</v>
       </c>
       <c r="T17" s="3">
-        <v>4.9445683999999996</v>
+        <v>9.7944429999999869</v>
       </c>
       <c r="U17" s="3">
         <v>166.82148999999998</v>
@@ -1991,19 +1942,19 @@
         <v>18.336808999999999</v>
       </c>
       <c r="W17" s="3">
-        <v>2860.5675430000001</v>
+        <v>2860.5675427000001</v>
       </c>
       <c r="X17" s="3">
         <v>193.2789555</v>
       </c>
       <c r="Y17" s="3">
-        <v>3260.9852850000002</v>
+        <v>3260.9852852000004</v>
       </c>
       <c r="Z17" s="3">
-        <v>7086.6795199999997</v>
-      </c>
-    </row>
-    <row r="18" spans="1:26" ht="15">
+        <v>7086.6795204</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -2062,7 +2013,7 @@
         <v>0</v>
       </c>
       <c r="T18" s="3">
-        <v>7.8731062000000005</v>
+        <v>43.963066600000005</v>
       </c>
       <c r="U18" s="3">
         <v>80.391941200000005</v>
@@ -2080,10 +2031,10 @@
         <v>950.86800999999991</v>
       </c>
       <c r="Z18" s="3">
-        <v>2169.6094739999999</v>
-      </c>
-    </row>
-    <row r="19" spans="1:26" ht="15">
+        <v>2169.6094736</v>
+      </c>
+    </row>
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -2139,10 +2090,10 @@
         <v>137.6097413</v>
       </c>
       <c r="S19" s="3">
-        <v>5.2191095000000001</v>
+        <v>0</v>
       </c>
       <c r="T19" s="3">
-        <v>54.61827370000001</v>
+        <v>75.391438300000146</v>
       </c>
       <c r="U19" s="3">
         <v>688.01730750000024</v>
@@ -2160,10 +2111,10 @@
         <v>1723.2436400000001</v>
       </c>
       <c r="Z19" s="3">
-        <v>3583.1484220000002</v>
-      </c>
-    </row>
-    <row r="20" spans="1:26" ht="15">
+        <v>3583.1484222999998</v>
+      </c>
+    </row>
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -2222,7 +2173,7 @@
         <v>0</v>
       </c>
       <c r="T20" s="3">
-        <v>61.358889599999998</v>
+        <v>72.049859099999978</v>
       </c>
       <c r="U20" s="3">
         <v>157.95744209999998</v>
@@ -2231,7 +2182,7 @@
         <v>44.725983300000003</v>
       </c>
       <c r="W20" s="3">
-        <v>1698.87898</v>
+        <v>1698.8789804</v>
       </c>
       <c r="X20" s="3">
         <v>80.494960699999993</v>
@@ -2240,10 +2191,10 @@
         <v>2365.39264</v>
       </c>
       <c r="Z20" s="3">
-        <v>5146.6092120000003</v>
-      </c>
-    </row>
-    <row r="21" spans="1:26" ht="15">
+        <v>5146.6092123999997</v>
+      </c>
+    </row>
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -2302,7 +2253,7 @@
         <v>0</v>
       </c>
       <c r="T21" s="3">
-        <v>58.052700399999992</v>
+        <v>63.231074399999962</v>
       </c>
       <c r="U21" s="3">
         <v>163.52343659999997</v>
@@ -2320,10 +2271,10 @@
         <v>993.89731000000006</v>
       </c>
       <c r="Z21" s="3">
-        <v>3410.5409369999998</v>
-      </c>
-    </row>
-    <row r="22" spans="1:26" ht="15">
+        <v>3410.5409368999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -2379,10 +2330,10 @@
         <v>61.899456200000003</v>
       </c>
       <c r="S22" s="3">
-        <v>10.560469700000001</v>
+        <v>0</v>
       </c>
       <c r="T22" s="3">
-        <v>26.424697799999997</v>
+        <v>54.23946519999997</v>
       </c>
       <c r="U22" s="3">
         <v>176.03653249999996</v>
@@ -2391,7 +2342,7 @@
         <v>38.092775500000002</v>
       </c>
       <c r="W22" s="3">
-        <v>2469.5193949999998</v>
+        <v>2469.5193951000001</v>
       </c>
       <c r="X22" s="3">
         <v>303.32530700000001</v>
@@ -2400,10 +2351,10 @@
         <v>2931.6890399999997</v>
       </c>
       <c r="Z22" s="3">
-        <v>4073.6389389999999</v>
-      </c>
-    </row>
-    <row r="23" spans="1:26" ht="15">
+        <v>4073.6389387999998</v>
+      </c>
+    </row>
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -2450,7 +2401,7 @@
         <v>4070.857852600001</v>
       </c>
       <c r="P23" s="3">
-        <v>820.63263319999965</v>
+        <v>820.6326332999995</v>
       </c>
       <c r="Q23" s="3">
         <v>31.385704000000004</v>
@@ -2459,19 +2410,19 @@
         <v>5.0850289999999996</v>
       </c>
       <c r="S23" s="3">
-        <v>1.6454440000000001</v>
+        <v>0</v>
       </c>
       <c r="T23" s="3">
-        <v>0.1710931</v>
+        <v>38.807798699999978</v>
       </c>
       <c r="U23" s="3">
         <v>75.278531699999988</v>
       </c>
       <c r="V23" s="3">
-        <v>116.3221818</v>
+        <v>116.32218189999999</v>
       </c>
       <c r="W23" s="3">
-        <v>5574.5211319999999</v>
+        <v>5574.5211322000005</v>
       </c>
       <c r="X23" s="3">
         <v>296.75909769999998</v>
@@ -2480,10 +2431,10 @@
         <v>5549.8929099999996</v>
       </c>
       <c r="Z23" s="3">
-        <v>6724.9257729999999</v>
-      </c>
-    </row>
-    <row r="24" spans="1:26" ht="15">
+        <v>6724.9257727000004</v>
+      </c>
+    </row>
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -2539,10 +2490,10 @@
         <v>4.6391985</v>
       </c>
       <c r="S24" s="3">
-        <v>12.786744000000001</v>
+        <v>0</v>
       </c>
       <c r="T24" s="3">
-        <v>14.143408700000002</v>
+        <v>32.798222700000018</v>
       </c>
       <c r="U24" s="3">
         <v>105.57776360000003</v>
@@ -2551,7 +2502,7 @@
         <v>33.975614800000002</v>
       </c>
       <c r="W24" s="3">
-        <v>1496.805249</v>
+        <v>1496.8052484999998</v>
       </c>
       <c r="X24" s="3">
         <v>105.5772726</v>
@@ -2560,10 +2511,10 @@
         <v>1719.621191</v>
       </c>
       <c r="Z24" s="3">
-        <v>3197.6853040000001</v>
-      </c>
-    </row>
-    <row r="25" spans="1:26" ht="15">
+        <v>3197.6853039000002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -2622,7 +2573,7 @@
         <v>0</v>
       </c>
       <c r="T25" s="3">
-        <v>7.3277083999999988</v>
+        <v>8.0540273999999989</v>
       </c>
       <c r="U25" s="3">
         <v>17.959651399999998</v>
@@ -2640,10 +2591,10 @@
         <v>513.80994999999996</v>
       </c>
       <c r="Z25" s="3">
-        <v>2488.336217</v>
-      </c>
-    </row>
-    <row r="26" spans="1:26" ht="15">
+        <v>2488.3362173999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -2699,10 +2650,10 @@
         <v>19.607319799999999</v>
       </c>
       <c r="S26" s="3">
-        <v>6.8319599999999996</v>
+        <v>0</v>
       </c>
       <c r="T26" s="3">
-        <v>9.5855040999999996</v>
+        <v>16.417464100000004</v>
       </c>
       <c r="U26" s="3">
         <v>46.586112700000001</v>
@@ -2711,19 +2662,19 @@
         <v>13.3466001</v>
       </c>
       <c r="W26" s="3">
-        <v>1391.472348</v>
+        <v>1391.4723478999999</v>
       </c>
       <c r="X26" s="3">
         <v>69.285299199999997</v>
       </c>
       <c r="Y26" s="3">
-        <v>1192.655278</v>
+        <v>1192.6552781</v>
       </c>
       <c r="Z26" s="3">
-        <v>5475.565517</v>
-      </c>
-    </row>
-    <row r="27" spans="1:26" ht="15">
+        <v>5475.5655167000004</v>
+      </c>
+    </row>
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -2773,37 +2724,37 @@
         <v>180.05286450000011</v>
       </c>
       <c r="Q27" s="3">
-        <v>19.1349482</v>
+        <v>28.801575800000002</v>
       </c>
       <c r="R27" s="3">
-        <v>29.846677500000002</v>
+        <v>32.187247500000005</v>
       </c>
       <c r="S27" s="3">
         <v>0</v>
       </c>
       <c r="T27" s="3">
-        <v>31.938939299999998</v>
+        <v>68.133291600000007</v>
       </c>
       <c r="U27" s="3">
         <v>140.06921490000002</v>
       </c>
       <c r="V27" s="3">
-        <v>120.3969408</v>
+        <v>143.3512384</v>
       </c>
       <c r="W27" s="3">
-        <v>2069.926406</v>
+        <v>2069.9264056000002</v>
       </c>
       <c r="X27" s="3">
         <v>63.218927999999998</v>
       </c>
       <c r="Y27" s="3">
-        <v>1642.9992200000002</v>
+        <v>1642.9992199000001</v>
       </c>
       <c r="Z27" s="3">
-        <v>5702.3282909999998</v>
-      </c>
-    </row>
-    <row r="28" spans="1:26" ht="15">
+        <v>5725.2830000000004</v>
+      </c>
+    </row>
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -2820,7 +2771,7 @@
         <v>3022.0342828000003</v>
       </c>
       <c r="F28" s="3">
-        <v>128.00999999999999</v>
+        <v>128.01</v>
       </c>
       <c r="G28" s="3">
         <v>3357.9162567000003</v>
@@ -2862,7 +2813,7 @@
         <v>0</v>
       </c>
       <c r="T28" s="3">
-        <v>22.011908199999997</v>
+        <v>31.494367499999999</v>
       </c>
       <c r="U28" s="3">
         <v>116.31125819999998</v>
@@ -2871,7 +2822,7 @@
         <v>139.5354998</v>
       </c>
       <c r="W28" s="3">
-        <v>1417.9613409999999</v>
+        <v>1417.9613412000001</v>
       </c>
       <c r="X28" s="3">
         <v>30.204251500000002</v>
@@ -2880,10 +2831,10 @@
         <v>2725.5114899999999</v>
       </c>
       <c r="Z28" s="3">
-        <v>5085.1007600000003</v>
-      </c>
-    </row>
-    <row r="29" spans="1:26" ht="15">
+        <v>5085.1007598000006</v>
+      </c>
+    </row>
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -2930,7 +2881,7 @@
         <v>2093.6943012999996</v>
       </c>
       <c r="P29" s="3">
-        <v>116.60185680000008</v>
+        <v>122.57478890000016</v>
       </c>
       <c r="Q29" s="3">
         <v>81.877869899999993</v>
@@ -2942,28 +2893,28 @@
         <v>0</v>
       </c>
       <c r="T29" s="3">
-        <v>8.7828929999999996</v>
+        <v>9.8019412000000017</v>
       </c>
       <c r="U29" s="3">
         <v>97.205871299999998</v>
       </c>
       <c r="V29" s="3">
-        <v>106.50962720000001</v>
+        <v>112.48255929999999</v>
       </c>
       <c r="W29" s="3">
-        <v>3173.504938</v>
+        <v>3173.5049380999999</v>
       </c>
       <c r="X29" s="3">
         <v>298.4732128</v>
       </c>
       <c r="Y29" s="3">
-        <v>2375.8238429999997</v>
+        <v>2375.8238425</v>
       </c>
       <c r="Z29" s="3">
-        <v>5936.1474840000001</v>
-      </c>
-    </row>
-    <row r="30" spans="1:26" ht="15">
+        <v>5942.12</v>
+      </c>
+    </row>
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -3022,7 +2973,7 @@
         <v>0</v>
       </c>
       <c r="T30" s="3">
-        <v>16.334318400000001</v>
+        <v>16.598054600000001</v>
       </c>
       <c r="U30" s="3">
         <v>63.4667879</v>
@@ -3031,7 +2982,7 @@
         <v>21.174385700000002</v>
       </c>
       <c r="W30" s="3">
-        <v>2146.4609310000001</v>
+        <v>2146.4609307999999</v>
       </c>
       <c r="X30" s="3">
         <v>60.485998600000002</v>
@@ -3040,10 +2991,10 @@
         <v>680.00280320000002</v>
       </c>
       <c r="Z30" s="3">
-        <v>6352.6267230000003</v>
-      </c>
-    </row>
-    <row r="31" spans="1:26" ht="15">
+        <v>6352.6267232999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>29</v>
       </c>
@@ -3102,7 +3053,7 @@
         <v>0</v>
       </c>
       <c r="T31" s="3">
-        <v>3.5234754000000001</v>
+        <v>56.033147500000013</v>
       </c>
       <c r="U31" s="3">
         <v>76.646223800000016</v>
@@ -3111,19 +3062,19 @@
         <v>69.113226799999993</v>
       </c>
       <c r="W31" s="3">
-        <v>2058.5580360000004</v>
+        <v>2058.5580355000002</v>
       </c>
       <c r="X31" s="3">
         <v>467.83135729999998</v>
       </c>
       <c r="Y31" s="3">
-        <v>1187.7480739999999</v>
+        <v>1187.7480744</v>
       </c>
       <c r="Z31" s="3">
-        <v>5012.615648</v>
-      </c>
-    </row>
-    <row r="32" spans="1:26" ht="15">
+        <v>5012.6156477000004</v>
+      </c>
+    </row>
+    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>30</v>
       </c>
@@ -3182,7 +3133,7 @@
         <v>0</v>
       </c>
       <c r="T32" s="3">
-        <v>1.4597673000000002</v>
+        <v>12.096429399999989</v>
       </c>
       <c r="U32" s="3">
         <v>73.970474699999983</v>
@@ -3200,10 +3151,10 @@
         <v>1512.0142499999999</v>
       </c>
       <c r="Z32" s="3">
-        <v>4782.6752820000002</v>
-      </c>
-    </row>
-    <row r="33" spans="1:26" ht="15">
+        <v>4782.6752815999998</v>
+      </c>
+    </row>
+    <row r="33" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -3259,10 +3210,10 @@
         <v>0</v>
       </c>
       <c r="S33" s="3">
-        <v>26.5</v>
+        <v>0</v>
       </c>
       <c r="T33" s="3">
-        <v>0</v>
+        <v>73.255698200000012</v>
       </c>
       <c r="U33" s="3">
         <v>73.255698200000012</v>
@@ -3271,7 +3222,7 @@
         <v>130.09267670000003</v>
       </c>
       <c r="W33" s="3">
-        <v>2294.6477150000001</v>
+        <v>2294.6477147000001</v>
       </c>
       <c r="X33" s="3">
         <v>725.32718560000001</v>
@@ -3280,10 +3231,10 @@
         <v>2424.7858000000001</v>
       </c>
       <c r="Z33" s="3">
-        <v>9187.4276890000001</v>
-      </c>
-    </row>
-    <row r="34" spans="1:26" ht="15">
+        <v>9187.4276884999999</v>
+      </c>
+    </row>
+    <row r="34" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>32</v>
       </c>
@@ -3342,7 +3293,7 @@
         <v>0</v>
       </c>
       <c r="T34" s="3">
-        <v>11.5104525</v>
+        <v>36.340688799999995</v>
       </c>
       <c r="U34" s="3">
         <v>93.794522000000001</v>
@@ -3351,19 +3302,19 @@
         <v>92.636170199999981</v>
       </c>
       <c r="W34" s="3">
-        <v>2106.1729989999999</v>
+        <v>2106.1729989</v>
       </c>
       <c r="X34" s="3">
         <v>199.57281259999999</v>
       </c>
       <c r="Y34" s="3">
-        <v>1007.0485359999999</v>
+        <v>1007.0485355000001</v>
       </c>
       <c r="Z34" s="3">
-        <v>5676.9830400000001</v>
-      </c>
-    </row>
-    <row r="35" spans="1:26" ht="15">
+        <v>5676.9830401999998</v>
+      </c>
+    </row>
+    <row r="35" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>33</v>
       </c>
@@ -3419,10 +3370,10 @@
         <v>1.6011369000000002</v>
       </c>
       <c r="S35" s="3">
-        <v>1.9272116999999997</v>
+        <v>0</v>
       </c>
       <c r="T35" s="3">
-        <v>15.158252900000003</v>
+        <v>19.855547099999992</v>
       </c>
       <c r="U35" s="3">
         <v>70.950319099999987</v>
@@ -3431,7 +3382,7 @@
         <v>20.178865699999996</v>
       </c>
       <c r="W35" s="3">
-        <v>1131.2421949999998</v>
+        <v>1131.2421950999999</v>
       </c>
       <c r="X35" s="3">
         <v>28.598458300000001</v>
@@ -3443,7 +3394,7 @@
         <v>4141.2187600000007</v>
       </c>
     </row>
-    <row r="36" spans="1:26" ht="15">
+    <row r="36" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>34</v>
       </c>
@@ -3502,7 +3453,7 @@
         <v>0</v>
       </c>
       <c r="T36" s="3">
-        <v>25.918280300000003</v>
+        <v>41.460799200000004</v>
       </c>
       <c r="U36" s="3">
         <v>118.3884377</v>
@@ -3511,19 +3462,19 @@
         <v>24.956009399999999</v>
       </c>
       <c r="W36" s="3">
-        <v>1854.2715730000002</v>
+        <v>1854.2715734000001</v>
       </c>
       <c r="X36" s="3">
         <v>138.8100101</v>
       </c>
       <c r="Y36" s="3">
-        <v>1319.064396</v>
+        <v>1319.0643956000001</v>
       </c>
       <c r="Z36" s="3">
-        <v>4721.7629189999998</v>
-      </c>
-    </row>
-    <row r="37" spans="1:26" ht="15">
+        <v>4721.7629190999996</v>
+      </c>
+    </row>
+    <row r="37" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>35</v>
       </c>
@@ -3540,7 +3491,7 @@
         <v>5973.5879711999996</v>
       </c>
       <c r="F37" s="3">
-        <v>46.390000000000001</v>
+        <v>46.39</v>
       </c>
       <c r="G37" s="3">
         <v>6133.1747166000005</v>
@@ -3582,7 +3533,7 @@
         <v>0</v>
       </c>
       <c r="T37" s="3">
-        <v>90.295765700000004</v>
+        <v>95.793565699999988</v>
       </c>
       <c r="U37" s="3">
         <v>111.9952562</v>
@@ -3591,7 +3542,7 @@
         <v>34.144373000000002</v>
       </c>
       <c r="W37" s="3">
-        <v>1952.026562</v>
+        <v>1952.0265624000001</v>
       </c>
       <c r="X37" s="3">
         <v>55.065093499999996</v>
@@ -3600,10 +3551,10 @@
         <v>941.73615000000007</v>
       </c>
       <c r="Z37" s="3">
-        <v>7074.7780940000002</v>
-      </c>
-    </row>
-    <row r="38" spans="1:26" ht="15">
+        <v>7074.7780942000009</v>
+      </c>
+    </row>
+    <row r="38" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>36</v>
       </c>
@@ -3659,10 +3610,10 @@
         <v>17.0235059</v>
       </c>
       <c r="S38" s="3">
-        <v>3.6279050000000002</v>
+        <v>0</v>
       </c>
       <c r="T38" s="3">
-        <v>7.5750043000000007</v>
+        <v>33.265486900000006</v>
       </c>
       <c r="U38" s="3">
         <v>58.296162800000005</v>
@@ -3677,13 +3628,13 @@
         <v>55.166861900000001</v>
       </c>
       <c r="Y38" s="3">
-        <v>1315.925414</v>
+        <v>1315.9254136</v>
       </c>
       <c r="Z38" s="3">
         <v>4944.5416279999999</v>
       </c>
     </row>
-    <row r="39" spans="1:26" ht="15">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>37</v>
       </c>
@@ -3739,10 +3690,10 @@
         <v>24.711157400000001</v>
       </c>
       <c r="S39" s="3">
-        <v>6.7602400000000005</v>
+        <v>0</v>
       </c>
       <c r="T39" s="3">
-        <v>16.731183100000003</v>
+        <v>29.530392899999995</v>
       </c>
       <c r="U39" s="3">
         <v>127.9841263</v>
@@ -3751,7 +3702,7 @@
         <v>14.590363900000002</v>
       </c>
       <c r="W39" s="3">
-        <v>2352.4711870000001</v>
+        <v>2352.4711864999999</v>
       </c>
       <c r="X39" s="3">
         <v>37.785236699999999</v>
@@ -3760,10 +3711,10 @@
         <v>2536.0147699999998</v>
       </c>
       <c r="Z39" s="3">
-        <v>9388.6687679999995</v>
-      </c>
-    </row>
-    <row r="40" spans="1:26" ht="15">
+        <v>9388.6687676000001</v>
+      </c>
+    </row>
+    <row r="40" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>38</v>
       </c>
@@ -3819,10 +3770,10 @@
         <v>0</v>
       </c>
       <c r="S40" s="3">
-        <v>5.3106719999999994</v>
+        <v>0</v>
       </c>
       <c r="T40" s="3">
-        <v>1.5803601999999999</v>
+        <v>6.8910321999999971</v>
       </c>
       <c r="U40" s="3">
         <v>48.677827199999996</v>
@@ -3831,7 +3782,7 @@
         <v>25.7614087</v>
       </c>
       <c r="W40" s="3">
-        <v>1791.6122250000001</v>
+        <v>1791.6122248000001</v>
       </c>
       <c r="X40" s="3">
         <v>125.20396860000001</v>
@@ -3843,7 +3794,7 @@
         <v>6079.8179319999999</v>
       </c>
     </row>
-    <row r="41" spans="1:26" ht="15">
+    <row r="41" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>39</v>
       </c>
@@ -3899,10 +3850,10 @@
         <v>1.2785888000000001</v>
       </c>
       <c r="S41" s="3">
-        <v>4.5497225000000006</v>
+        <v>0</v>
       </c>
       <c r="T41" s="3">
-        <v>1.2321900000000001</v>
+        <v>10.021912500000001</v>
       </c>
       <c r="U41" s="3">
         <v>11.300501300000001</v>
@@ -3920,10 +3871,10 @@
         <v>969.97782440000015</v>
       </c>
       <c r="Z41" s="3">
-        <v>3306.42625</v>
-      </c>
-    </row>
-    <row r="42" spans="1:26" ht="15">
+        <v>3306.4262501000003</v>
+      </c>
+    </row>
+    <row r="42" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>40</v>
       </c>
@@ -3982,7 +3933,7 @@
         <v>0</v>
       </c>
       <c r="T42" s="3">
-        <v>10.6543838</v>
+        <v>11.669971200000003</v>
       </c>
       <c r="U42" s="3">
         <v>34.203050100000006</v>
@@ -4000,10 +3951,10 @@
         <v>529.05953999999997</v>
       </c>
       <c r="Z42" s="3">
-        <v>4083.1091290000004</v>
-      </c>
-    </row>
-    <row r="43" spans="1:26" ht="15">
+        <v>4083.1091289000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>41</v>
       </c>
@@ -4059,10 +4010,10 @@
         <v>9.3407478000000008</v>
       </c>
       <c r="S43" s="3">
-        <v>4.1195132000000001</v>
+        <v>0</v>
       </c>
       <c r="T43" s="3">
-        <v>4.9588768999999999</v>
+        <v>10.070434499999999</v>
       </c>
       <c r="U43" s="3">
         <v>19.4111823</v>
@@ -4071,7 +4022,7 @@
         <v>10.914444500000002</v>
       </c>
       <c r="W43" s="3">
-        <v>1292.0388210000001</v>
+        <v>1292.0388214000002</v>
       </c>
       <c r="X43" s="3">
         <v>43.358786700000003</v>
@@ -4080,10 +4031,10 @@
         <v>1194.0866099999998</v>
       </c>
       <c r="Z43" s="3">
-        <v>7065.1887099999994</v>
-      </c>
-    </row>
-    <row r="44" spans="1:26" ht="15">
+        <v>7065.1887096999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>42</v>
       </c>
@@ -4142,7 +4093,7 @@
         <v>0</v>
       </c>
       <c r="T44" s="3">
-        <v>24.770247000000001</v>
+        <v>25.551606700000004</v>
       </c>
       <c r="U44" s="3">
         <v>82.762124099999994</v>
@@ -4160,10 +4111,10 @@
         <v>267.78130999999996</v>
       </c>
       <c r="Z44" s="3">
-        <v>3050.0277510000001</v>
-      </c>
-    </row>
-    <row r="45" spans="1:26" ht="15">
+        <v>3050.0277513999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>43</v>
       </c>
@@ -4219,10 +4170,10 @@
         <v>19.521562200000002</v>
       </c>
       <c r="S45" s="3">
-        <v>7.6747472999999999</v>
+        <v>0</v>
       </c>
       <c r="T45" s="3">
-        <v>46.017994699999996</v>
+        <v>61.973445099999999</v>
       </c>
       <c r="U45" s="3">
         <v>93.684979400000003</v>
@@ -4231,7 +4182,7 @@
         <v>18.473657500000002</v>
       </c>
       <c r="W45" s="3">
-        <v>1530.3605190000001</v>
+        <v>1530.3605191000001</v>
       </c>
       <c r="X45" s="3">
         <v>76.896851400000003</v>
@@ -4240,10 +4191,10 @@
         <v>566.51165000000003</v>
       </c>
       <c r="Z45" s="3">
-        <v>6974.3728790000005</v>
-      </c>
-    </row>
-    <row r="46" spans="1:26" ht="15">
+        <v>6974.3728786999991</v>
+      </c>
+    </row>
+    <row r="46" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>44</v>
       </c>
@@ -4299,10 +4250,10 @@
         <v>27.533695400000003</v>
       </c>
       <c r="S46" s="3">
-        <v>3.7915859000000003</v>
+        <v>0</v>
       </c>
       <c r="T46" s="3">
-        <v>36.612861800000005</v>
+        <v>46.559903100000007</v>
       </c>
       <c r="U46" s="3">
         <v>85.11001850000001</v>
@@ -4311,7 +4262,7 @@
         <v>0</v>
       </c>
       <c r="W46" s="3">
-        <v>1456.729016</v>
+        <v>1456.7290163999999</v>
       </c>
       <c r="X46" s="3">
         <v>97.414919300000008</v>
@@ -4320,10 +4271,10 @@
         <v>954.28537000000006</v>
       </c>
       <c r="Z46" s="3">
-        <v>4453.7328070000003</v>
-      </c>
-    </row>
-    <row r="47" spans="1:26" ht="15">
+        <v>4453.7328068999996</v>
+      </c>
+    </row>
+    <row r="47" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>45</v>
       </c>
@@ -4382,7 +4333,7 @@
         <v>0</v>
       </c>
       <c r="T47" s="3">
-        <v>41.401750999999997</v>
+        <v>41.401751000000012</v>
       </c>
       <c r="U47" s="3">
         <v>121.78118710000001</v>
@@ -4391,7 +4342,7 @@
         <v>7.5577758999999993</v>
       </c>
       <c r="W47" s="3">
-        <v>1089.702448</v>
+        <v>1089.7024479000002</v>
       </c>
       <c r="X47" s="3">
         <v>84.359020799999996</v>
@@ -4400,10 +4351,10 @@
         <v>461.2789113</v>
       </c>
       <c r="Z47" s="3">
-        <v>5657.6867670000001</v>
-      </c>
-    </row>
-    <row r="48" spans="1:26" ht="15">
+        <v>5657.6867671</v>
+      </c>
+    </row>
+    <row r="48" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>46</v>
       </c>
@@ -4420,7 +4371,7 @@
         <v>4485.0454298000004</v>
       </c>
       <c r="F48" s="3">
-        <v>60.390000000000001</v>
+        <v>60.39</v>
       </c>
       <c r="G48" s="3">
         <v>4764.4601698000006</v>
@@ -4462,7 +4413,7 @@
         <v>0</v>
       </c>
       <c r="T48" s="3">
-        <v>13.304180299999999</v>
+        <v>13.304180299999997</v>
       </c>
       <c r="U48" s="3">
         <v>32.765794799999995</v>
@@ -4471,7 +4422,7 @@
         <v>0</v>
       </c>
       <c r="W48" s="3">
-        <v>1180.424454</v>
+        <v>1180.4244538</v>
       </c>
       <c r="X48" s="3">
         <v>64.506394700000001</v>
@@ -4480,10 +4431,10 @@
         <v>1060.8694399999999</v>
       </c>
       <c r="Z48" s="3">
-        <v>5571.2141750000001</v>
-      </c>
-    </row>
-    <row r="49" spans="1:26" ht="15">
+        <v>5571.2141748999993</v>
+      </c>
+    </row>
+    <row r="49" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>47</v>
       </c>
@@ -4542,7 +4493,7 @@
         <v>0</v>
       </c>
       <c r="T49" s="3">
-        <v>1.3818482999999999</v>
+        <v>1.3818483000000019</v>
       </c>
       <c r="U49" s="3">
         <v>44.837444900000001</v>
@@ -4560,10 +4511,10 @@
         <v>677.56930999999997</v>
       </c>
       <c r="Z49" s="3">
-        <v>3150.6981000000001</v>
-      </c>
-    </row>
-    <row r="50" spans="1:26" ht="15">
+        <v>3150.6980997000001</v>
+      </c>
+    </row>
+    <row r="50" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
         <v>48</v>
       </c>
@@ -4619,10 +4570,10 @@
         <v>9.5861867000000007</v>
       </c>
       <c r="S50" s="3">
-        <v>1.6375066</v>
+        <v>0</v>
       </c>
       <c r="T50" s="3">
-        <v>10.1807152</v>
+        <v>11.818221799999996</v>
       </c>
       <c r="U50" s="3">
         <v>23.730660999999998</v>
@@ -4640,10 +4591,10 @@
         <v>140.86893000000001</v>
       </c>
       <c r="Z50" s="3">
-        <v>2042.3327899999999</v>
-      </c>
-    </row>
-    <row r="51" spans="1:26" ht="15">
+        <v>2042.3327901</v>
+      </c>
+    </row>
+    <row r="51" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
         <v>49</v>
       </c>
@@ -4660,7 +4611,7 @@
         <v>2698.4488386000003</v>
       </c>
       <c r="F51" s="3">
-        <v>194.38999999999999</v>
+        <v>194.39</v>
       </c>
       <c r="G51" s="3">
         <v>2933.6188386000003</v>
@@ -4699,10 +4650,10 @@
         <v>15.115076800000002</v>
       </c>
       <c r="S51" s="3">
-        <v>2.1658548999999998</v>
+        <v>0</v>
       </c>
       <c r="T51" s="3">
-        <v>23.255296699999999</v>
+        <v>33.130161600000008</v>
       </c>
       <c r="U51" s="3">
         <v>48.245238400000012</v>
@@ -4720,10 +4671,10 @@
         <v>236.26172990000001</v>
       </c>
       <c r="Z51" s="3">
-        <v>3540.5448659999997</v>
-      </c>
-    </row>
-    <row r="52" spans="1:26" ht="15">
+        <v>3540.5448655999999</v>
+      </c>
+    </row>
+    <row r="52" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A52" s="1">
         <v>50</v>
       </c>
@@ -4779,10 +4730,10 @@
         <v>0</v>
       </c>
       <c r="S52" s="3">
-        <v>8.5297951999999988</v>
+        <v>0</v>
       </c>
       <c r="T52" s="3">
-        <v>0</v>
+        <v>21.445843400000001</v>
       </c>
       <c r="U52" s="3">
         <v>21.445843400000001</v>
@@ -4800,10 +4751,10 @@
         <v>478.83888790000003</v>
       </c>
       <c r="Z52" s="3">
-        <v>1957.5401979999999</v>
-      </c>
-    </row>
-    <row r="53" spans="1:26" ht="15">
+        <v>1957.5401976999999</v>
+      </c>
+    </row>
+    <row r="53" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
         <v>51</v>
       </c>
@@ -4871,7 +4822,7 @@
         <v>0</v>
       </c>
       <c r="W53" s="3">
-        <v>1390.655773</v>
+        <v>1390.6557734</v>
       </c>
       <c r="X53" s="3">
         <v>50.545893300000003</v>
@@ -4880,10 +4831,10 @@
         <v>1083.90707</v>
       </c>
       <c r="Z53" s="3">
-        <v>4452.4752429999999</v>
-      </c>
-    </row>
-    <row r="54" spans="1:26" ht="15">
+        <v>4452.4752427000003</v>
+      </c>
+    </row>
+    <row r="54" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A54" s="1">
         <v>52</v>
       </c>
@@ -4939,10 +4890,10 @@
         <v>56.988525799999998</v>
       </c>
       <c r="S54" s="3">
-        <v>17.867341400000001</v>
+        <v>0</v>
       </c>
       <c r="T54" s="3">
-        <v>41.306686499999998</v>
+        <v>67.52185320000001</v>
       </c>
       <c r="U54" s="3">
         <v>143.36286490000001</v>
@@ -4963,7 +4914,7 @@
         <v>3586.513074</v>
       </c>
     </row>
-    <row r="55" spans="1:26" ht="15">
+    <row r="55" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A55" s="1">
         <v>53</v>
       </c>
@@ -5022,7 +4973,7 @@
         <v>0</v>
       </c>
       <c r="T55" s="3">
-        <v>34.556551999999996</v>
+        <v>36.65588300000001</v>
       </c>
       <c r="U55" s="3">
         <v>126.11336870000001</v>
@@ -5031,7 +4982,7 @@
         <v>16.0862026</v>
       </c>
       <c r="W55" s="3">
-        <v>1413.90453</v>
+        <v>1413.9045297</v>
       </c>
       <c r="X55" s="3">
         <v>58.061769399999996</v>
@@ -5043,7 +4994,7 @@
         <v>2661.7354780000001</v>
       </c>
     </row>
-    <row r="56" spans="1:26" ht="15">
+    <row r="56" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
         <v>54</v>
       </c>
@@ -5123,8 +5074,15 @@
         <v>15.008009999999999</v>
       </c>
     </row>
+    <row r="57" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="S57" s="3">
+        <v>0</v>
+      </c>
+      <c r="T57" s="3">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>